<commit_message>
Add Appointment Letter generation with Annexure C salary breakdown and dual document portal
</commit_message>
<xml_diff>
--- a/sample_candidates.xlsx
+++ b/sample_candidates.xlsx
@@ -47,8 +47,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
   </fills>
@@ -450,22 +450,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="53" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,44 +506,69 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Offer Date</t>
+          <t>Issue Date</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Document Type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Work Location</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Reporting Location</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Reporting Time</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>HR Signatory</t>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Probation Period</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Signatory Name</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Signatory Title</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Abhishek Rajput</t>
+          <t>Roshan Machindra Mokal</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -548,150 +578,200 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Chief Production Master</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>5000000</v>
+        <v>1020000</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Fifty Lakh only/-</t>
+          <t>Ten Lakh Twenty Thousand only/-</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>20-10-2026</t>
+          <t>05-Oct-2026</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>05-Oct-2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Marine Drive Patna, Bihar 843323</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>+91 9267778873</t>
+          <t>1007, tower 5, cluster 5, Blossom City, Near Rayan International School, Runwal Garden City, Usarghar, Dombivli 421204</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>abhi@gmail.com</t>
+          <t>+91 9022229535</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Nanakramguda</t>
+          <t>roshan0mahendra@gmail.com</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>10.00 AM</t>
+          <t>Mumbai - CPU</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Sruti Associate - HR</t>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>10:00 a.m.</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Three (3) months</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Harley’s India Private Limited</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>K Harishanker Goud</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Authorized Signatory</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Priya Sharma</t>
+          <t>Abhishek Rajput</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Ms.</t>
+          <t>Mr.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Senior Full Stack Developer</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1800000</v>
+        <v>5000000</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Eighteen Lakh only/-</t>
+          <t>Fifty Lakh only/-</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>01-11-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Plot 42, Hitech City, Hyderabad, Telangana 500081</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>+91 9876501234</t>
+          <t>Marine Drive Patna, Bihar 843323</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>priya.sharma@example.com</t>
+          <t>+91 9267778873</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
+          <t>abhi@gmail.com</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad - Nanakramguda</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
           <t>Nanakramguda</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>10.00 AM</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Three (3) months</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>HARLEY INDIA PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Sruti Associate - HR</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Associate - HR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Rahul Verma</t>
+          <t>Priya Sharma</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Mr.</t>
+          <t>Ms.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Marketing Manager</t>
+          <t>Senior Full Stack Developer</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1200000</v>
+        <v>1800000</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Twelve Lakh only/-</t>
+          <t>Eighteen Lakh only/-</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>15-11-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -701,32 +781,57 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Flat 301, Whitefield, Bangalore, Karnataka 560066</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>+91 9123456789</t>
+          <t>Plot 42, Hitech City, Hyderabad, Telangana 500081</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>rahul.verma@example.com</t>
+          <t>+91 9876501234</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
+          <t>priya.sharma@example.com</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad - Nanakramguda</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
           <t>Nanakramguda</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>10.00 AM</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Sruti Associate - HR</t>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Three (3) months</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Harley’s India Private Limited</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>K Harishanker Goud</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Authorized Signatory</t>
         </is>
       </c>
     </row>

</xml_diff>